<commit_message>
Major Change : Phase 1A
Refactors staff dashboards into role-based administrator/supervisor views and adds shared submission eligibility logic, enforcement middleware, and transaction-safe enrollment/submission flows. This also updates the UI branding to e-Pasca, adds sidebar work-count widgets and theme styling, renames the submission eligibility screens, and includes focused feature coverage for eligibility, bulk actions, and historical access rules.
</commit_message>
<xml_diff>
--- a/public/assets/excel-template/e-PGS_STAFF_REGISTRATION_TEMPLATE.xlsx
+++ b/public/assets/excel-template/e-PGS_STAFF_REGISTRATION_TEMPLATE.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\User\Desktop\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\laragon\www\fyp-project\public\assets\excel-template\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A0CD5725-0BE2-4C28-93D1-253CD108D7CD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7CF2A4AF-2A1D-4C09-ACB1-AC33A5B225E3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{7205C628-2ECF-4FA1-95A4-550522F5FFD8}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="15720" xr2:uid="{7205C628-2ECF-4FA1-95A4-550522F5FFD8}"/>
   </bookViews>
   <sheets>
     <sheet name="e-PGS Staff Registration" sheetId="1" r:id="rId1"/>
@@ -66,10 +66,10 @@
     <t>EX. 01113097495</t>
   </si>
   <si>
-    <t>EX. SE, DB, AI</t>
-  </si>
-  <si>
-    <t>EX. COMM, LECT, TDP, DEAN</t>
+    <t>COMM</t>
+  </si>
+  <si>
+    <t>FTMKSE</t>
   </si>
 </sst>
 </file>
@@ -168,12 +168,11 @@
         <u val="none"/>
         <vertAlign val="baseline"/>
         <sz val="11"/>
-        <color theme="1"/>
+        <color rgb="FF000000"/>
         <name val="Calibri"/>
         <family val="2"/>
         <scheme val="minor"/>
       </font>
-      <numFmt numFmtId="30" formatCode="@"/>
     </dxf>
     <dxf>
       <font>
@@ -205,11 +204,12 @@
         <u val="none"/>
         <vertAlign val="baseline"/>
         <sz val="11"/>
-        <color rgb="FF000000"/>
+        <color theme="1"/>
         <name val="Calibri"/>
         <family val="2"/>
         <scheme val="minor"/>
       </font>
+      <numFmt numFmtId="30" formatCode="@"/>
     </dxf>
     <dxf>
       <font>
@@ -328,9 +328,9 @@
     <tableColumn id="1" xr3:uid="{002C293F-6CD3-43DB-8B76-2B45D8CD0133}" name="staff_id" dataDxfId="5"/>
     <tableColumn id="2" xr3:uid="{DB84A27A-0797-4B18-9545-949A00AC4C8F}" name="staff_name" dataDxfId="4"/>
     <tableColumn id="3" xr3:uid="{A216302B-9EF0-4830-97A8-6B0FF133C2A2}" name="staff_email" dataDxfId="3" dataCellStyle="Hyperlink"/>
-    <tableColumn id="4" xr3:uid="{66572F2B-D61C-4A5D-B912-65213296A877}" name="staff_phoneno" dataDxfId="0"/>
-    <tableColumn id="5" xr3:uid="{8D7FC06C-E2FB-4648-86A0-142CE8C5F69A}" name="staff_department" dataDxfId="2"/>
-    <tableColumn id="6" xr3:uid="{E8F7AD5E-D903-4183-B7D5-35BEC0A95353}" name="staff_role" dataDxfId="1"/>
+    <tableColumn id="4" xr3:uid="{66572F2B-D61C-4A5D-B912-65213296A877}" name="staff_phoneno" dataDxfId="2"/>
+    <tableColumn id="5" xr3:uid="{8D7FC06C-E2FB-4648-86A0-142CE8C5F69A}" name="staff_department" dataDxfId="1"/>
+    <tableColumn id="6" xr3:uid="{E8F7AD5E-D903-4183-B7D5-35BEC0A95353}" name="staff_role" dataDxfId="0"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleLight1" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -634,18 +634,18 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{40EAC937-8C1A-415E-B4D3-7BDDC8094CE5}">
   <dimension ref="A1:F2"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="15.77734375" style="1" customWidth="1"/>
-    <col min="2" max="2" width="62.21875" style="1" customWidth="1"/>
-    <col min="3" max="3" width="23.33203125" style="1" customWidth="1"/>
+    <col min="1" max="1" width="15.7109375" style="1" customWidth="1"/>
+    <col min="2" max="2" width="62.28515625" style="1" customWidth="1"/>
+    <col min="3" max="3" width="23.28515625" style="1" customWidth="1"/>
     <col min="4" max="4" width="20" style="7" customWidth="1"/>
-    <col min="5" max="5" width="19.5546875" style="1" customWidth="1"/>
-    <col min="6" max="6" width="25.21875" style="1" customWidth="1"/>
-    <col min="7" max="16384" width="8.88671875" style="1"/>
+    <col min="5" max="5" width="19.5703125" style="1" customWidth="1"/>
+    <col min="6" max="6" width="25.28515625" style="1" customWidth="1"/>
+    <col min="7" max="16384" width="8.85546875" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" s="3" customFormat="1" ht="23.4" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:6" s="3" customFormat="1" ht="23.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
@@ -665,7 +665,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A2" s="1" t="s">
         <v>6</v>
       </c>
@@ -679,13 +679,21 @@
         <v>9</v>
       </c>
       <c r="E2" s="5" t="s">
+        <v>11</v>
+      </c>
+      <c r="F2" s="5" t="s">
         <v>10</v>
-      </c>
-      <c r="F2" s="5" t="s">
-        <v>11</v>
       </c>
     </row>
   </sheetData>
+  <dataValidations count="2">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="F2" xr:uid="{E39E9890-67A7-4D03-AC97-E6BEAE37C1CD}">
+      <formula1>"COMM,LECT,TDP,DEAN"</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="E2" xr:uid="{5419FF6E-F514-49FE-B178-0770178DE3C1}">
+      <formula1>"FTMKAI,FTMKSE,FTMKDB,FAIXAI"</formula1>
+    </dataValidation>
+  </dataValidations>
   <hyperlinks>
     <hyperlink ref="C2" r:id="rId1" display="maslita@utem.edu.my" xr:uid="{09BD03F4-E134-4C57-BA13-729CEF0C2C42}"/>
   </hyperlinks>

</xml_diff>